<commit_message>
Refocus project scope for progress meeting
</commit_message>
<xml_diff>
--- a/department-course-clustering/data/raw/collection_checklist.xlsx
+++ b/department-course-clustering/data/raw/collection_checklist.xlsx
@@ -640,7 +640,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>GitHub external 2개 권장과목 파일 자동 매칭; rows=263</t>
+          <t>GitHub external 2개 권장과목 파일 자동 매칭; rows=258</t>
         </is>
       </c>
     </row>
@@ -677,7 +677,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>GitHub external 2개 권장과목 파일 자동 매칭; rows=256</t>
+          <t>GitHub external 2개 권장과목 파일 자동 매칭; rows=280</t>
         </is>
       </c>
     </row>
@@ -825,7 +825,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>GitHub external 2개 권장과목 파일 자동 매칭; rows=271</t>
+          <t>GitHub external 2개 권장과목 파일 자동 매칭; rows=166</t>
         </is>
       </c>
     </row>
@@ -862,7 +862,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>GitHub external 2개 권장과목 파일 자동 매칭; rows=211</t>
+          <t>GitHub external 2개 권장과목 파일 자동 매칭; rows=163</t>
         </is>
       </c>
     </row>
@@ -936,7 +936,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>GitHub external 2개 권장과목 파일 자동 매칭; rows=236</t>
+          <t>GitHub external 2개 권장과목 파일 자동 매칭; rows=276</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>GitHub external 2개 권장과목 파일 자동 매칭; rows=96</t>
+          <t>GitHub external 2개 권장과목 파일 자동 매칭; rows=47</t>
         </is>
       </c>
     </row>
@@ -1047,7 +1047,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>GitHub external 2개 권장과목 파일 자동 매칭; rows=599</t>
+          <t>GitHub external 2개 권장과목 파일 자동 매칭; rows=555</t>
         </is>
       </c>
     </row>
@@ -1494,7 +1494,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=13; units=건축공학과; 건축학과</t>
+          <t>자동 매칭 rows=36; units=건축공학과; 건축학과</t>
         </is>
       </c>
     </row>
@@ -1536,7 +1536,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=6; units=국어국문학과</t>
+          <t>자동 매칭 rows=14; units=국어국문학과</t>
         </is>
       </c>
     </row>
@@ -1578,7 +1578,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=5; units=심리학과</t>
+          <t>자동 매칭 rows=14; units=심리학과</t>
         </is>
       </c>
     </row>
@@ -1620,7 +1620,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=12; units=기계공학부</t>
+          <t>자동 매칭 rows=30; units=기계공학부</t>
         </is>
       </c>
     </row>
@@ -1662,7 +1662,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=9; units=화학과</t>
+          <t>자동 매칭 rows=23; units=화학과</t>
         </is>
       </c>
     </row>
@@ -1704,7 +1704,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=7; units=산업공학과</t>
+          <t>자동 매칭 rows=16; units=산업공학과</t>
         </is>
       </c>
     </row>
@@ -1788,7 +1788,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=10; units=조선해양공학과</t>
+          <t>자동 매칭 rows=24; units=조선해양공학과</t>
         </is>
       </c>
     </row>
@@ -1830,7 +1830,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=7; units=의예과</t>
+          <t>자동 매칭 rows=19; units=의예과</t>
         </is>
       </c>
     </row>
@@ -1872,7 +1872,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=9; units=수학과</t>
+          <t>자동 매칭 rows=22; units=수학과</t>
         </is>
       </c>
     </row>
@@ -1914,7 +1914,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=10; units=경영학과</t>
+          <t>자동 매칭 rows=24; units=경영학과</t>
         </is>
       </c>
     </row>
@@ -1956,7 +1956,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=4; units=약학부</t>
+          <t>자동 매칭 rows=9; units=약학부</t>
         </is>
       </c>
     </row>
@@ -1998,7 +1998,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=5; units=사회학과</t>
+          <t>자동 매칭 rows=14; units=사회학과</t>
         </is>
       </c>
     </row>
@@ -2040,7 +2040,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=8; units=경제학부</t>
+          <t>자동 매칭 rows=22; units=경제학부</t>
         </is>
       </c>
     </row>
@@ -2082,7 +2082,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=7; units=생명과학과</t>
+          <t>자동 매칭 rows=20; units=생명과학과</t>
         </is>
       </c>
     </row>
@@ -2124,7 +2124,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=3; units=미디어커뮤니케이션학과</t>
+          <t>자동 매칭 rows=8; units=미디어커뮤니케이션학과</t>
         </is>
       </c>
     </row>
@@ -2166,7 +2166,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=8; units=화공생명공학과</t>
+          <t>자동 매칭 rows=22; units=화공생명공학과</t>
         </is>
       </c>
     </row>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=5; units=디자인학과-애니메이션전공; 실내환경디자인학과</t>
+          <t>자동 매칭 rows=13; units=디자인학과-애니메이션전공; 실내환경디자인학과</t>
         </is>
       </c>
     </row>
@@ -2250,7 +2250,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=5; units=식품영양학과</t>
+          <t>자동 매칭 rows=14; units=식품영양학과</t>
         </is>
       </c>
     </row>
@@ -2292,7 +2292,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=9; units=간호학과</t>
+          <t>자동 매칭 rows=24; units=간호학과</t>
         </is>
       </c>
     </row>
@@ -2376,7 +2376,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=6; units=사학과</t>
+          <t>자동 매칭 rows=15; units=사학과</t>
         </is>
       </c>
     </row>
@@ -2418,7 +2418,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=7; units=통계학과</t>
+          <t>자동 매칭 rows=16; units=통계학과</t>
         </is>
       </c>
     </row>
@@ -4518,7 +4518,7 @@
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=24; units=건축학과; 스마트시티건축공학과</t>
+          <t>자동 매칭 rows=60; units=건축학과; 스마트시티건축공학과</t>
         </is>
       </c>
     </row>
@@ -4560,7 +4560,7 @@
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=12; units=국어국문학과</t>
+          <t>자동 매칭 rows=30; units=국어국문학과</t>
         </is>
       </c>
     </row>
@@ -4602,7 +4602,7 @@
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=9; units=심리학과</t>
+          <t>자동 매칭 rows=22; units=심리학과</t>
         </is>
       </c>
     </row>
@@ -4644,7 +4644,7 @@
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=12; units=기계공학부</t>
+          <t>자동 매칭 rows=30; units=기계공학부</t>
         </is>
       </c>
     </row>
@@ -4686,7 +4686,7 @@
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=27; units=생물환경화학과; 생화학과; 화학과</t>
+          <t>자동 매칭 rows=68; units=생물환경화학과; 생화학과; 화학과</t>
         </is>
       </c>
     </row>
@@ -4770,7 +4770,7 @@
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=12; units=신소재공학과</t>
+          <t>자동 매칭 rows=30; units=신소재공학과</t>
         </is>
       </c>
     </row>
@@ -4854,7 +4854,7 @@
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=18; units=의예과</t>
+          <t>자동 매칭 rows=46; units=의예과</t>
         </is>
       </c>
     </row>
@@ -4896,7 +4896,7 @@
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=12; units=수학과</t>
+          <t>자동 매칭 rows=30; units=수학과</t>
         </is>
       </c>
     </row>
@@ -4938,7 +4938,7 @@
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=12; units=경영학부</t>
+          <t>자동 매칭 rows=30; units=경영학부</t>
         </is>
       </c>
     </row>
@@ -4980,7 +4980,7 @@
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=9; units=약학과</t>
+          <t>자동 매칭 rows=22; units=약학과</t>
         </is>
       </c>
     </row>
@@ -5022,7 +5022,7 @@
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=12; units=사회학과</t>
+          <t>자동 매칭 rows=30; units=사회학과</t>
         </is>
       </c>
     </row>
@@ -5064,7 +5064,7 @@
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=12; units=경제학과</t>
+          <t>자동 매칭 rows=30; units=경제학과</t>
         </is>
       </c>
     </row>
@@ -5106,7 +5106,7 @@
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=9; units=미생물분자생명과학과</t>
+          <t>자동 매칭 rows=22; units=미생물분자생명과학과</t>
         </is>
       </c>
     </row>
@@ -5148,7 +5148,7 @@
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=12; units=언론정보학과</t>
+          <t>자동 매칭 rows=30; units=언론정보학과</t>
         </is>
       </c>
     </row>
@@ -5190,7 +5190,7 @@
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=12; units=응용화학공학과</t>
+          <t>자동 매칭 rows=30; units=응용화학공학과</t>
         </is>
       </c>
     </row>
@@ -5274,7 +5274,7 @@
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=12; units=식품영양학과</t>
+          <t>자동 매칭 rows=30; units=식품영양학과</t>
         </is>
       </c>
     </row>
@@ -5316,7 +5316,7 @@
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=15; units=간호학과</t>
+          <t>자동 매칭 rows=38; units=간호학과</t>
         </is>
       </c>
     </row>
@@ -5358,7 +5358,7 @@
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=24; units=전기공학과; 전자공학과</t>
+          <t>자동 매칭 rows=60; units=전기공학과; 전자공학과</t>
         </is>
       </c>
     </row>
@@ -5400,7 +5400,7 @@
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=24; units=국사학과; 사학과</t>
+          <t>자동 매칭 rows=60; units=국사학과; 사학과</t>
         </is>
       </c>
     </row>
@@ -5442,7 +5442,7 @@
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=9; units=정보통계학과</t>
+          <t>자동 매칭 rows=22; units=정보통계학과</t>
         </is>
       </c>
     </row>
@@ -5526,7 +5526,7 @@
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=14; units=건축공학과; 건축학과</t>
+          <t>자동 매칭 rows=42; units=건축공학과; 건축학과</t>
         </is>
       </c>
     </row>
@@ -5568,7 +5568,7 @@
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=8; units=국어국문학과</t>
+          <t>자동 매칭 rows=24; units=국어국문학과</t>
         </is>
       </c>
     </row>
@@ -5610,7 +5610,7 @@
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=8; units=심리학과</t>
+          <t>자동 매칭 rows=24; units=심리학과</t>
         </is>
       </c>
     </row>
@@ -5652,7 +5652,7 @@
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=8; units=기계공학부</t>
+          <t>자동 매칭 rows=24; units=기계공학부</t>
         </is>
       </c>
     </row>
@@ -5694,7 +5694,7 @@
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=52; units=공업화학과; 독일언어문화학과; 러시아언어문화학과; 생화학과; 프랑스언어문화학과; 화학과; 환경생명화학과</t>
+          <t>자동 매칭 rows=156; units=공업화학과; 독일언어문화학과; 러시아언어문화학과; 생화학과; 프랑스언어문화학과; 화학과; 환경생명화학과</t>
         </is>
       </c>
     </row>
@@ -5778,7 +5778,7 @@
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=8; units=신소재공학과</t>
+          <t>자동 매칭 rows=24; units=신소재공학과</t>
         </is>
       </c>
     </row>
@@ -5862,7 +5862,7 @@
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=16; units=식물의학과; 의예과</t>
+          <t>자동 매칭 rows=48; units=식물의학과; 의예과</t>
         </is>
       </c>
     </row>
@@ -5904,7 +5904,7 @@
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=6; units=수학과</t>
+          <t>자동 매칭 rows=18; units=수학과</t>
         </is>
       </c>
     </row>
@@ -5946,7 +5946,7 @@
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=16; units=경영학부; 국제경영학과</t>
+          <t>자동 매칭 rows=48; units=경영학부; 국제경영학과</t>
         </is>
       </c>
     </row>
@@ -5988,7 +5988,7 @@
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=4; units=약학과; 제약학과</t>
+          <t>자동 매칭 rows=12; units=약학과; 제약학과</t>
         </is>
       </c>
     </row>
@@ -6030,7 +6030,7 @@
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=8; units=사회학과</t>
+          <t>자동 매칭 rows=24; units=사회학과</t>
         </is>
       </c>
     </row>
@@ -6072,7 +6072,7 @@
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=8; units=경제학과</t>
+          <t>자동 매칭 rows=24; units=경제학과</t>
         </is>
       </c>
     </row>
@@ -6198,7 +6198,7 @@
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=6; units=화학공학과</t>
+          <t>자동 매칭 rows=18; units=화학공학과</t>
         </is>
       </c>
     </row>
@@ -6282,7 +6282,7 @@
       </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=4; units=식품영양학과</t>
+          <t>자동 매칭 rows=12; units=식품영양학과</t>
         </is>
       </c>
     </row>
@@ -6324,7 +6324,7 @@
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=8; units=간호학과</t>
+          <t>자동 매칭 rows=24; units=간호학과</t>
         </is>
       </c>
     </row>
@@ -6366,7 +6366,7 @@
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=8; units=전자공학과</t>
+          <t>자동 매칭 rows=24; units=전자공학과</t>
         </is>
       </c>
     </row>
@@ -6408,7 +6408,7 @@
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=12; units=고고미술사학과; 사학과</t>
+          <t>자동 매칭 rows=36; units=고고미술사학과; 사학과</t>
         </is>
       </c>
     </row>
@@ -6450,7 +6450,7 @@
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=8; units=정보통계학과</t>
+          <t>자동 매칭 rows=24; units=정보통계학과</t>
         </is>
       </c>
     </row>
@@ -6492,7 +6492,7 @@
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=10; units=컴퓨터공학과</t>
+          <t>자동 매칭 rows=30; units=컴퓨터공학과</t>
         </is>
       </c>
     </row>
@@ -8550,7 +8550,7 @@
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=4; units=건축학과</t>
+          <t>자동 매칭 rows=10; units=건축학과</t>
         </is>
       </c>
     </row>
@@ -8592,7 +8592,7 @@
       </c>
       <c r="H171" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=4; units=국어국문학과</t>
+          <t>자동 매칭 rows=14; units=국어국문학과</t>
         </is>
       </c>
     </row>
@@ -8634,7 +8634,7 @@
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=3; units=심리학과</t>
+          <t>자동 매칭 rows=10; units=심리학과</t>
         </is>
       </c>
     </row>
@@ -8676,7 +8676,7 @@
       </c>
       <c r="H173" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=9; units=기계공학부; 생물산업기계공학과; 스마트에너지기계공학과</t>
+          <t>자동 매칭 rows=30; units=기계공학부; 생물산업기계공학과; 스마트에너지기계공학과</t>
         </is>
       </c>
     </row>
@@ -8718,7 +8718,7 @@
       </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=8; units=화학과; 환경생명화학과</t>
+          <t>자동 매칭 rows=26; units=화학과; 환경생명화학과</t>
         </is>
       </c>
     </row>
@@ -8844,7 +8844,7 @@
       </c>
       <c r="H177" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=3; units=조선해양공학과</t>
+          <t>자동 매칭 rows=10; units=조선해양공학과</t>
         </is>
       </c>
     </row>
@@ -8886,7 +8886,7 @@
       </c>
       <c r="H178" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=13; units=식물의학과; 의예과; 해양식품생명의학부</t>
+          <t>자동 매칭 rows=44; units=식물의학과; 의예과; 해양식품생명의학부</t>
         </is>
       </c>
     </row>
@@ -8970,7 +8970,7 @@
       </c>
       <c r="H180" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=8; units=경영학부; 해양수산경영학과</t>
+          <t>자동 매칭 rows=26; units=경영학부; 해양수산경영학과</t>
         </is>
       </c>
     </row>
@@ -9012,7 +9012,7 @@
       </c>
       <c r="H181" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=6; units=약학과</t>
+          <t>자동 매칭 rows=18; units=약학과</t>
         </is>
       </c>
     </row>
@@ -9054,7 +9054,7 @@
       </c>
       <c r="H182" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=3; units=사회학과</t>
+          <t>자동 매칭 rows=10; units=사회학과</t>
         </is>
       </c>
     </row>
@@ -9096,7 +9096,7 @@
       </c>
       <c r="H183" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=6; units=경제학부</t>
+          <t>자동 매칭 rows=20; units=경제학부</t>
         </is>
       </c>
     </row>
@@ -9138,7 +9138,7 @@
       </c>
       <c r="H184" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=8; units=생명과학부; 해양생명과학과</t>
+          <t>자동 매칭 rows=28; units=생명과학부; 해양생명과학과</t>
         </is>
       </c>
     </row>
@@ -9180,7 +9180,7 @@
       </c>
       <c r="H185" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=3; units=미디어커뮤니케이션학과</t>
+          <t>자동 매칭 rows=10; units=미디어커뮤니케이션학과</t>
         </is>
       </c>
     </row>
@@ -9222,7 +9222,7 @@
       </c>
       <c r="H186" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=4; units=화학공학과</t>
+          <t>자동 매칭 rows=12; units=화학공학과</t>
         </is>
       </c>
     </row>
@@ -9306,7 +9306,7 @@
       </c>
       <c r="H188" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=6; units=식품영양학과</t>
+          <t>자동 매칭 rows=20; units=식품영양학과</t>
         </is>
       </c>
     </row>
@@ -9348,7 +9348,7 @@
       </c>
       <c r="H189" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=6; units=간호학과</t>
+          <t>자동 매칭 rows=20; units=간호학과</t>
         </is>
       </c>
     </row>
@@ -9390,7 +9390,7 @@
       </c>
       <c r="H190" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=3; units=전기공학과</t>
+          <t>자동 매칭 rows=10; units=전기공학과</t>
         </is>
       </c>
     </row>
@@ -9432,7 +9432,7 @@
       </c>
       <c r="H191" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=4; units=사학과</t>
+          <t>자동 매칭 rows=12; units=사학과</t>
         </is>
       </c>
     </row>
@@ -9464,7 +9464,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>없음</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -9474,7 +9474,7 @@
       </c>
       <c r="H192" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=3; units=정보통계학과</t>
+          <t>자동 매칭 rows=12; units=정보통계학과</t>
         </is>
       </c>
     </row>
@@ -9516,7 +9516,7 @@
       </c>
       <c r="H193" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=4; units=컴퓨터공학부</t>
+          <t>자동 매칭 rows=14; units=컴퓨터공학부</t>
         </is>
       </c>
     </row>
@@ -9894,7 +9894,7 @@
       </c>
       <c r="H202" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=6; units=의예과</t>
+          <t>자동 매칭 rows=16; units=의예과</t>
         </is>
       </c>
     </row>
@@ -10356,7 +10356,7 @@
       </c>
       <c r="H213" s="2" t="inlineStr">
         <is>
-          <t>자동 매칭 rows=9; units=간호학과</t>
+          <t>자동 매칭 rows=23; units=간호학과</t>
         </is>
       </c>
     </row>
@@ -11554,27 +11554,27 @@
       </c>
       <c r="D242" s="2" t="inlineStr">
         <is>
-          <t>미확인/없음</t>
+          <t>있음</t>
         </is>
       </c>
       <c r="E242" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="G242" s="2" t="inlineStr">
         <is>
-          <t>필요</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="H242" s="2" t="inlineStr">
         <is>
-          <t>원본 컷 파일에서 자동 매칭 실패 또는 해당 모집단위 없음</t>
+          <t>자동 매칭 rows=28; units=건축공학과; 건축학과</t>
         </is>
       </c>
     </row>
@@ -11680,27 +11680,27 @@
       </c>
       <c r="D245" s="2" t="inlineStr">
         <is>
-          <t>미확인/없음</t>
+          <t>있음</t>
         </is>
       </c>
       <c r="E245" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F245" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="G245" s="2" t="inlineStr">
         <is>
-          <t>필요</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="H245" s="2" t="inlineStr">
         <is>
-          <t>원본 컷 파일에서 자동 매칭 실패 또는 해당 모집단위 없음</t>
+          <t>자동 매칭 rows=17; units=기계공학과</t>
         </is>
       </c>
     </row>
@@ -11722,27 +11722,27 @@
       </c>
       <c r="D246" s="2" t="inlineStr">
         <is>
-          <t>미확인/없음</t>
+          <t>있음</t>
         </is>
       </c>
       <c r="E246" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F246" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="G246" s="2" t="inlineStr">
         <is>
-          <t>필요</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="H246" s="2" t="inlineStr">
         <is>
-          <t>원본 컷 파일에서 자동 매칭 실패 또는 해당 모집단위 없음</t>
+          <t>자동 매칭 rows=14; units=화학과</t>
         </is>
       </c>
     </row>
@@ -11806,27 +11806,27 @@
       </c>
       <c r="D248" s="2" t="inlineStr">
         <is>
-          <t>미확인/없음</t>
+          <t>있음</t>
         </is>
       </c>
       <c r="E248" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F248" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="G248" s="2" t="inlineStr">
         <is>
-          <t>필요</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="H248" s="2" t="inlineStr">
         <is>
-          <t>원본 컷 파일에서 자동 매칭 실패 또는 해당 모집단위 없음</t>
+          <t>자동 매칭 rows=17; units=신소재공학과</t>
         </is>
       </c>
     </row>
@@ -11848,27 +11848,27 @@
       </c>
       <c r="D249" s="2" t="inlineStr">
         <is>
-          <t>미확인/없음</t>
+          <t>있음</t>
         </is>
       </c>
       <c r="E249" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F249" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="G249" s="2" t="inlineStr">
         <is>
-          <t>필요</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="H249" s="2" t="inlineStr">
         <is>
-          <t>원본 컷 파일에서 자동 매칭 실패 또는 해당 모집단위 없음</t>
+          <t>자동 매칭 rows=14; units=조선해양공학과</t>
         </is>
       </c>
     </row>
@@ -11890,27 +11890,27 @@
       </c>
       <c r="D250" s="2" t="inlineStr">
         <is>
-          <t>미확인/없음</t>
+          <t>있음</t>
         </is>
       </c>
       <c r="E250" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="G250" s="2" t="inlineStr">
         <is>
-          <t>필요</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="H250" s="2" t="inlineStr">
         <is>
-          <t>원본 컷 파일에서 자동 매칭 실패 또는 해당 모집단위 없음</t>
+          <t>자동 매칭 rows=7; units=의예과</t>
         </is>
       </c>
     </row>
@@ -11932,27 +11932,27 @@
       </c>
       <c r="D251" s="2" t="inlineStr">
         <is>
-          <t>미확인/없음</t>
+          <t>있음</t>
         </is>
       </c>
       <c r="E251" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F251" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="G251" s="2" t="inlineStr">
         <is>
-          <t>필요</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="H251" s="2" t="inlineStr">
         <is>
-          <t>원본 컷 파일에서 자동 매칭 실패 또는 해당 모집단위 없음</t>
+          <t>자동 매칭 rows=14; units=정보수학과</t>
         </is>
       </c>
     </row>
@@ -11974,27 +11974,27 @@
       </c>
       <c r="D252" s="2" t="inlineStr">
         <is>
-          <t>미확인/없음</t>
+          <t>있음</t>
         </is>
       </c>
       <c r="E252" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F252" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="G252" s="2" t="inlineStr">
         <is>
-          <t>필요</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="H252" s="2" t="inlineStr">
         <is>
-          <t>원본 컷 파일에서 자동 매칭 실패 또는 해당 모집단위 없음</t>
+          <t>자동 매칭 rows=34; units=경영학과; 관광경영학과</t>
         </is>
       </c>
     </row>
@@ -12100,27 +12100,27 @@
       </c>
       <c r="D255" s="2" t="inlineStr">
         <is>
-          <t>미확인/없음</t>
+          <t>있음</t>
         </is>
       </c>
       <c r="E255" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F255" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="G255" s="2" t="inlineStr">
         <is>
-          <t>필요</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="H255" s="2" t="inlineStr">
         <is>
-          <t>원본 컷 파일에서 자동 매칭 실패 또는 해당 모집단위 없음</t>
+          <t>자동 매칭 rows=14; units=경제학과</t>
         </is>
       </c>
     </row>
@@ -12184,27 +12184,27 @@
       </c>
       <c r="D257" s="2" t="inlineStr">
         <is>
-          <t>미확인/없음</t>
+          <t>있음</t>
         </is>
       </c>
       <c r="E257" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F257" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="G257" s="2" t="inlineStr">
         <is>
-          <t>필요</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="H257" s="2" t="inlineStr">
         <is>
-          <t>원본 컷 파일에서 자동 매칭 실패 또는 해당 모집단위 없음</t>
+          <t>자동 매칭 rows=14; units=미디어커뮤니케이션학과</t>
         </is>
       </c>
     </row>
@@ -12226,27 +12226,27 @@
       </c>
       <c r="D258" s="2" t="inlineStr">
         <is>
-          <t>미확인/없음</t>
+          <t>있음</t>
         </is>
       </c>
       <c r="E258" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F258" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="G258" s="2" t="inlineStr">
         <is>
-          <t>필요</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="H258" s="2" t="inlineStr">
         <is>
-          <t>원본 컷 파일에서 자동 매칭 실패 또는 해당 모집단위 없음</t>
+          <t>자동 매칭 rows=17; units=화학공학과</t>
         </is>
       </c>
     </row>
@@ -12268,27 +12268,27 @@
       </c>
       <c r="D259" s="2" t="inlineStr">
         <is>
-          <t>미확인/없음</t>
+          <t>있음</t>
         </is>
       </c>
       <c r="E259" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F259" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="G259" s="2" t="inlineStr">
         <is>
-          <t>필요</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="H259" s="2" t="inlineStr">
         <is>
-          <t>원본 컷 파일에서 자동 매칭 실패 또는 해당 모집단위 없음</t>
+          <t>자동 매칭 rows=17; units=산업디자인학과; 패션디자인학과</t>
         </is>
       </c>
     </row>
@@ -12310,27 +12310,27 @@
       </c>
       <c r="D260" s="2" t="inlineStr">
         <is>
-          <t>미확인/없음</t>
+          <t>있음</t>
         </is>
       </c>
       <c r="E260" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F260" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="G260" s="2" t="inlineStr">
         <is>
-          <t>필요</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="H260" s="2" t="inlineStr">
         <is>
-          <t>원본 컷 파일에서 자동 매칭 실패 또는 해당 모집단위 없음</t>
+          <t>자동 매칭 rows=14; units=식품영양학과</t>
         </is>
       </c>
     </row>
@@ -12352,27 +12352,27 @@
       </c>
       <c r="D261" s="2" t="inlineStr">
         <is>
-          <t>미확인/없음</t>
+          <t>있음</t>
         </is>
       </c>
       <c r="E261" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F261" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="G261" s="2" t="inlineStr">
         <is>
-          <t>필요</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="H261" s="2" t="inlineStr">
         <is>
-          <t>원본 컷 파일에서 자동 매칭 실패 또는 해당 모집단위 없음</t>
+          <t>자동 매칭 rows=10; units=간호학과</t>
         </is>
       </c>
     </row>
@@ -12394,27 +12394,27 @@
       </c>
       <c r="D262" s="2" t="inlineStr">
         <is>
-          <t>미확인/없음</t>
+          <t>있음</t>
         </is>
       </c>
       <c r="E262" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F262" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="G262" s="2" t="inlineStr">
         <is>
-          <t>필요</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="H262" s="2" t="inlineStr">
         <is>
-          <t>원본 컷 파일에서 자동 매칭 실패 또는 해당 모집단위 없음</t>
+          <t>자동 매칭 rows=34; units=전기공학과; 전자공학과</t>
         </is>
       </c>
     </row>
@@ -12436,27 +12436,27 @@
       </c>
       <c r="D263" s="2" t="inlineStr">
         <is>
-          <t>미확인/없음</t>
+          <t>있음</t>
         </is>
       </c>
       <c r="E263" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F263" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="G263" s="2" t="inlineStr">
         <is>
-          <t>필요</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="H263" s="2" t="inlineStr">
         <is>
-          <t>원본 컷 파일에서 자동 매칭 실패 또는 해당 모집단위 없음</t>
+          <t>자동 매칭 rows=14; units=역사고고미술사학과</t>
         </is>
       </c>
     </row>
@@ -12520,27 +12520,27 @@
       </c>
       <c r="D265" s="2" t="inlineStr">
         <is>
-          <t>미확인/없음</t>
+          <t>있음</t>
         </is>
       </c>
       <c r="E265" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="F265" s="2" t="inlineStr">
         <is>
-          <t>미수집</t>
+          <t>완료</t>
         </is>
       </c>
       <c r="G265" s="2" t="inlineStr">
         <is>
-          <t>필요</t>
+          <t>아니오</t>
         </is>
       </c>
       <c r="H265" s="2" t="inlineStr">
         <is>
-          <t>원본 컷 파일에서 자동 매칭 실패 또는 해당 모집단위 없음</t>
+          <t>자동 매칭 rows=14; units=컴퓨터공학과</t>
         </is>
       </c>
     </row>

</xml_diff>